<commit_message>
feat: add storefront services and safe NDI inquiry
</commit_message>
<xml_diff>
--- a/application/tests/Fixtures/Ndi/stock_all_warehouses.xlsx
+++ b/application/tests/Fixtures/Ndi/stock_all_warehouses.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Article" sheetId="1" r:id="R178e9fd0fd694da5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Article" sheetId="1" r:id="R8783ebeff340408b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -392,19 +392,19 @@
         <x:v>0001234567890</x:v>
       </x:c>
       <x:c r="B2" s="26" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="C2" s="26" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="D2" s="26" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E2" s="26" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F2" s="26" t="n">
         <x:v>5</x:v>
-      </x:c>
-      <x:c r="C2" s="26" t="n">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="D2" s="26" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="E2" s="26" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="F2" s="26" t="n">
-        <x:v>0</x:v>
       </x:c>
       <x:c r="G2" s="26" t="n">
         <x:v>0</x:v>

</xml_diff>